<commit_message>
Corrected species names in dados.xlsx
</commit_message>
<xml_diff>
--- a/dados.xlsx
+++ b/dados.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/joaobiosmac/Desktop/R/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/joaobiosmac/Desktop/Trabalhos &amp; Repositórios/Artigos em Andamento/Paper Guariuma/Guariuma/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{237A569E-1327-5D47-A0FC-8369FF803EBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B4BF13B-292C-104E-BAB6-DCA249E04D97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="380" yWindow="620" windowWidth="28040" windowHeight="15240" xr2:uid="{542FE1DC-28D5-D64E-A92E-B09676E09D2F}"/>
   </bookViews>
@@ -76,9 +76,6 @@
     <t>Atlantirivulus santensis</t>
   </si>
   <si>
-    <t>Phalloceros sp.</t>
-  </si>
-  <si>
     <t>Hyphessobrycon boulengeri</t>
   </si>
   <si>
@@ -247,9 +244,6 @@
     <t>4.17</t>
   </si>
   <si>
-    <t>Characidium sp.</t>
-  </si>
-  <si>
     <t>24°00'05.0"S 46°32'59.0"W</t>
   </si>
   <si>
@@ -776,6 +770,12 @@
   </si>
   <si>
     <t>Coordenadas</t>
+  </si>
+  <si>
+    <t>Phalloceros circummontanus</t>
+  </si>
+  <si>
+    <t>Characidium lanei</t>
   </si>
 </sst>
 </file>
@@ -1174,7 +1174,9 @@
     <col min="13" max="13" width="19.5" customWidth="1"/>
     <col min="14" max="14" width="25.33203125" customWidth="1"/>
     <col min="15" max="15" width="23.83203125" customWidth="1"/>
-    <col min="16" max="23" width="25.33203125" customWidth="1"/>
+    <col min="16" max="16" width="25.33203125" customWidth="1"/>
+    <col min="17" max="17" width="27.5" customWidth="1"/>
+    <col min="18" max="23" width="25.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23" s="3" customFormat="1" x14ac:dyDescent="0.2">
@@ -1185,13 +1187,13 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>4</v>
@@ -1218,34 +1220,34 @@
         <v>11</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="O1" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="P1" s="2" t="s">
         <v>12</v>
       </c>
       <c r="Q1" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="R1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="S1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="S1" s="2" t="s">
-        <v>15</v>
-      </c>
       <c r="T1" s="2" t="s">
-        <v>70</v>
+        <v>246</v>
       </c>
       <c r="U1" s="2" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="V1" s="2" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="W1" s="2" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
     </row>
     <row r="2" spans="1:23" x14ac:dyDescent="0.2">
@@ -1253,10 +1255,10 @@
         <v>2025</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="D2" s="1">
         <v>1</v>
@@ -1265,13 +1267,13 @@
         <v>3</v>
       </c>
       <c r="F2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>18</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>19</v>
       </c>
       <c r="I2" s="1">
         <v>58</v>
@@ -1280,10 +1282,10 @@
         <v>33</v>
       </c>
       <c r="K2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="L2" s="1" t="s">
         <v>20</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>21</v>
       </c>
       <c r="M2" s="1">
         <v>21</v>
@@ -1292,7 +1294,7 @@
         <v>20</v>
       </c>
       <c r="O2" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="P2" s="1">
         <v>14</v>
@@ -1324,25 +1326,25 @@
         <v>2025</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="D3" s="1">
         <v>3</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F3" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="G3" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="H3" s="1" t="s">
         <v>28</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>29</v>
       </c>
       <c r="I3" s="1">
         <v>46</v>
@@ -1351,10 +1353,10 @@
         <v>23</v>
       </c>
       <c r="K3" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="L3" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="L3" s="1" t="s">
-        <v>31</v>
       </c>
       <c r="M3" s="1">
         <v>38</v>
@@ -1363,7 +1365,7 @@
         <v>3</v>
       </c>
       <c r="O3" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="P3" s="1">
         <v>6</v>
@@ -1395,25 +1397,25 @@
         <v>2025</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="D4" s="1">
         <v>4</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F4" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="G4" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="H4" s="1" t="s">
         <v>35</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>36</v>
       </c>
       <c r="I4" s="1">
         <v>32</v>
@@ -1422,7 +1424,7 @@
         <v>16</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="L4" s="1">
         <v>1</v>
@@ -1434,7 +1436,7 @@
         <v>3</v>
       </c>
       <c r="O4" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="P4" s="1">
         <v>3</v>
@@ -1466,25 +1468,25 @@
         <v>2025</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="D5" s="1">
         <v>5</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F5" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="G5" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="H5" s="1" t="s">
         <v>41</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>42</v>
       </c>
       <c r="I5" s="1">
         <v>60</v>
@@ -1493,10 +1495,10 @@
         <v>30</v>
       </c>
       <c r="K5" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="L5" s="1" t="s">
         <v>43</v>
-      </c>
-      <c r="L5" s="1" t="s">
-        <v>44</v>
       </c>
       <c r="M5" s="1">
         <v>34</v>
@@ -1505,7 +1507,7 @@
         <v>0</v>
       </c>
       <c r="O5" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="P5" s="1">
         <v>0</v>
@@ -1537,25 +1539,25 @@
         <v>2025</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="D6" s="1">
         <v>6</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F6" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G6" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="H6" s="1" t="s">
         <v>48</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>49</v>
       </c>
       <c r="I6" s="1">
         <v>137</v>
@@ -1564,10 +1566,10 @@
         <v>68</v>
       </c>
       <c r="K6" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="L6" s="1" t="s">
         <v>50</v>
-      </c>
-      <c r="L6" s="1" t="s">
-        <v>51</v>
       </c>
       <c r="M6" s="1">
         <v>56</v>
@@ -1576,7 +1578,7 @@
         <v>1</v>
       </c>
       <c r="O6" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="P6" s="1">
         <v>1</v>
@@ -1608,25 +1610,25 @@
         <v>2025</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="D7" s="1">
         <v>8</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F7" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="G7" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="G7" s="1" t="s">
+      <c r="H7" s="1" t="s">
         <v>56</v>
-      </c>
-      <c r="H7" s="1" t="s">
-        <v>57</v>
       </c>
       <c r="I7" s="1">
         <v>53</v>
@@ -1635,10 +1637,10 @@
         <v>26</v>
       </c>
       <c r="K7" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="L7" s="1" t="s">
         <v>58</v>
-      </c>
-      <c r="L7" s="1" t="s">
-        <v>59</v>
       </c>
       <c r="M7" s="1">
         <v>12</v>
@@ -1647,7 +1649,7 @@
         <v>0</v>
       </c>
       <c r="O7" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="P7" s="1">
         <v>2</v>
@@ -1679,25 +1681,25 @@
         <v>2025</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="D8" s="1">
         <v>10</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F8" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="G8" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="G8" s="1" t="s">
+      <c r="H8" s="1" t="s">
         <v>63</v>
-      </c>
-      <c r="H8" s="1" t="s">
-        <v>64</v>
       </c>
       <c r="I8" s="1">
         <v>112</v>
@@ -1709,7 +1711,7 @@
         <v>3</v>
       </c>
       <c r="L8" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="M8" s="1">
         <v>49</v>
@@ -1718,7 +1720,7 @@
         <v>0</v>
       </c>
       <c r="O8" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="P8" s="1">
         <v>0</v>
@@ -1750,25 +1752,25 @@
         <v>2025</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="D9" s="1">
         <v>11</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F9" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="G9" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="G9" s="1" t="s">
+      <c r="H9" s="1" t="s">
         <v>68</v>
-      </c>
-      <c r="H9" s="1" t="s">
-        <v>69</v>
       </c>
       <c r="I9" s="1">
         <v>51</v>
@@ -1789,7 +1791,7 @@
         <v>3</v>
       </c>
       <c r="O9" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="P9" s="1">
         <v>1</v>
@@ -1821,25 +1823,25 @@
         <v>2025</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="D10" s="1">
         <v>12</v>
       </c>
       <c r="E10" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="F10" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="G10" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="H10" s="1" t="s">
         <v>73</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="H10" s="1" t="s">
-        <v>75</v>
       </c>
       <c r="I10" s="1">
         <v>73</v>
@@ -1851,7 +1853,7 @@
         <v>10</v>
       </c>
       <c r="L10" s="1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="M10" s="1">
         <v>33</v>
@@ -1860,7 +1862,7 @@
         <v>0</v>
       </c>
       <c r="O10" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="P10" s="1">
         <v>3</v>
@@ -1892,25 +1894,25 @@
         <v>2025</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="D11" s="4">
         <v>13</v>
       </c>
       <c r="E11" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="G11" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="F11" s="4" t="s">
+      <c r="H11" s="4" t="s">
         <v>80</v>
-      </c>
-      <c r="G11" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="H11" s="4" t="s">
-        <v>82</v>
       </c>
       <c r="I11" s="4">
         <v>192</v>
@@ -1919,10 +1921,10 @@
         <v>96</v>
       </c>
       <c r="K11" s="4" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="L11" s="4" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="M11" s="4">
         <v>23</v>
@@ -1931,7 +1933,7 @@
         <v>0</v>
       </c>
       <c r="O11" s="4" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="P11" s="4">
         <v>1</v>
@@ -1963,25 +1965,25 @@
         <v>2025</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="D12" s="4">
         <v>14</v>
       </c>
       <c r="E12" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="G12" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="F12" s="4" t="s">
+      <c r="H12" s="4" t="s">
         <v>86</v>
-      </c>
-      <c r="G12" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="H12" s="4" t="s">
-        <v>88</v>
       </c>
       <c r="I12" s="4">
         <v>39</v>
@@ -1990,10 +1992,10 @@
         <v>20</v>
       </c>
       <c r="K12" s="4" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="L12" s="4" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="M12" s="4">
         <v>24</v>
@@ -2002,7 +2004,7 @@
         <v>3</v>
       </c>
       <c r="O12" s="4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="P12" s="4">
         <v>1</v>
@@ -2034,25 +2036,25 @@
         <v>2025</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="D13" s="4">
         <v>15</v>
       </c>
       <c r="E13" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="F13" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="F13" s="4" t="s">
+      <c r="G13" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="H13" s="4" t="s">
         <v>95</v>
-      </c>
-      <c r="G13" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="H13" s="4" t="s">
-        <v>97</v>
       </c>
       <c r="I13" s="4">
         <v>53</v>
@@ -2061,19 +2063,19 @@
         <v>27</v>
       </c>
       <c r="K13" s="4" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="L13" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="M13" s="4" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="N13" s="4">
         <v>0</v>
       </c>
       <c r="O13" s="4" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="P13" s="4">
         <v>0</v>
@@ -2105,25 +2107,25 @@
         <v>2025</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="D14" s="4">
         <v>16</v>
       </c>
       <c r="E14" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="F14" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="F14" s="4" t="s">
+      <c r="G14" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="H14" s="4" t="s">
         <v>102</v>
-      </c>
-      <c r="G14" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="H14" s="4" t="s">
-        <v>104</v>
       </c>
       <c r="I14" s="4">
         <v>84</v>
@@ -2132,10 +2134,10 @@
         <v>42</v>
       </c>
       <c r="K14" s="4" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="L14" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="M14" s="4">
         <v>34</v>
@@ -2144,7 +2146,7 @@
         <v>1</v>
       </c>
       <c r="O14" s="4" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="P14" s="4">
         <v>2</v>
@@ -2176,25 +2178,25 @@
         <v>2025</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="D15" s="4">
         <v>17</v>
       </c>
       <c r="E15" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="F15" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="F15" s="4" t="s">
+      <c r="G15" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="H15" s="4" t="s">
         <v>108</v>
-      </c>
-      <c r="G15" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="H15" s="4" t="s">
-        <v>110</v>
       </c>
       <c r="I15" s="4">
         <v>245</v>
@@ -2206,7 +2208,7 @@
         <v>4</v>
       </c>
       <c r="L15" s="4" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="M15" s="4">
         <v>31</v>
@@ -2215,7 +2217,7 @@
         <v>0</v>
       </c>
       <c r="O15" s="4" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="P15" s="4">
         <v>8</v>
@@ -2247,25 +2249,25 @@
         <v>2025</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="D16" s="4">
         <v>19</v>
       </c>
       <c r="E16" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="F16" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="F16" s="4" t="s">
-        <v>114</v>
-      </c>
       <c r="G16" s="4" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I16" s="4">
         <v>55</v>
@@ -2274,10 +2276,10 @@
         <v>27</v>
       </c>
       <c r="K16" s="4" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="L16" s="4" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="M16" s="4">
         <v>36</v>
@@ -2286,7 +2288,7 @@
         <v>2</v>
       </c>
       <c r="O16" s="4" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="P16" s="4">
         <v>2</v>
@@ -2318,25 +2320,25 @@
         <v>2025</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="D17" s="1">
         <v>20</v>
       </c>
       <c r="E17" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="H17" s="1" t="s">
         <v>119</v>
-      </c>
-      <c r="F17" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="G17" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="H17" s="1" t="s">
-        <v>121</v>
       </c>
       <c r="I17" s="1">
         <v>60</v>
@@ -2345,10 +2347,10 @@
         <v>29</v>
       </c>
       <c r="K17" s="1" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="L17" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="M17" s="1">
         <v>41</v>
@@ -2357,7 +2359,7 @@
         <v>2</v>
       </c>
       <c r="O17" s="1" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="P17" s="1">
         <v>0</v>
@@ -2389,25 +2391,25 @@
         <v>2025</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="D18" s="1">
         <v>21</v>
       </c>
       <c r="E18" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="G18" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="F18" s="1" t="s">
+      <c r="H18" s="1" t="s">
         <v>125</v>
-      </c>
-      <c r="G18" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="H18" s="1" t="s">
-        <v>127</v>
       </c>
       <c r="I18" s="1">
         <v>268</v>
@@ -2416,10 +2418,10 @@
         <v>134</v>
       </c>
       <c r="K18" s="1" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="L18" s="1" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="M18" s="1">
         <v>20</v>
@@ -2428,7 +2430,7 @@
         <v>0</v>
       </c>
       <c r="O18" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="P18" s="1">
         <v>6</v>
@@ -2460,25 +2462,25 @@
         <v>2025</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="D19" s="1">
         <v>22</v>
       </c>
       <c r="E19" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="G19" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="F19" s="1" t="s">
+      <c r="H19" s="1" t="s">
         <v>132</v>
-      </c>
-      <c r="G19" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="H19" s="1" t="s">
-        <v>134</v>
       </c>
       <c r="I19" s="1">
         <v>79</v>
@@ -2487,10 +2489,10 @@
         <v>40</v>
       </c>
       <c r="K19" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="L19" s="1" t="s">
         <v>135</v>
-      </c>
-      <c r="L19" s="1" t="s">
-        <v>137</v>
       </c>
       <c r="M19" s="1">
         <v>11</v>
@@ -2499,7 +2501,7 @@
         <v>0</v>
       </c>
       <c r="O19" s="1" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="P19" s="1">
         <v>2</v>
@@ -2531,25 +2533,25 @@
         <v>2025</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="D20" s="1">
         <v>23</v>
       </c>
       <c r="E20" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="F20" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="F20" s="1" t="s">
+      <c r="G20" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="H20" s="1" t="s">
         <v>142</v>
-      </c>
-      <c r="G20" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="H20" s="1" t="s">
-        <v>144</v>
       </c>
       <c r="I20" s="1">
         <v>75</v>
@@ -2558,10 +2560,10 @@
         <v>37</v>
       </c>
       <c r="K20" s="1" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="L20" s="1" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="M20" s="1">
         <v>29</v>
@@ -2570,7 +2572,7 @@
         <v>0</v>
       </c>
       <c r="O20" s="1" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="P20" s="1">
         <v>1</v>
@@ -2602,25 +2604,25 @@
         <v>2025</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="D21" s="1">
         <v>24</v>
       </c>
       <c r="E21" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="F21" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="F21" s="1" t="s">
+      <c r="G21" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="H21" s="1" t="s">
         <v>149</v>
-      </c>
-      <c r="G21" s="1" t="s">
-        <v>150</v>
-      </c>
-      <c r="H21" s="1" t="s">
-        <v>151</v>
       </c>
       <c r="I21" s="1">
         <v>99</v>
@@ -2629,10 +2631,10 @@
         <v>49</v>
       </c>
       <c r="K21" s="1" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="L21" s="1" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="M21" s="1">
         <v>22</v>
@@ -2641,7 +2643,7 @@
         <v>0</v>
       </c>
       <c r="O21" s="1" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="P21" s="1">
         <v>4</v>
@@ -2673,25 +2675,25 @@
         <v>2025</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="D22" s="1">
         <v>25</v>
       </c>
       <c r="E22" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="F22" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="F22" s="1" t="s">
+      <c r="G22" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="H22" s="1" t="s">
         <v>155</v>
-      </c>
-      <c r="G22" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="H22" s="1" t="s">
-        <v>157</v>
       </c>
       <c r="I22" s="1">
         <v>41</v>
@@ -2700,10 +2702,10 @@
         <v>21</v>
       </c>
       <c r="K22" s="1" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="L22" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="M22" s="1">
         <v>15</v>
@@ -2712,7 +2714,7 @@
         <v>0</v>
       </c>
       <c r="O22" s="1" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="P22" s="1">
         <v>4</v>
@@ -2744,22 +2746,22 @@
         <v>2025</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="D23" s="1">
         <v>26</v>
       </c>
       <c r="E23" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="F23" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="F23" s="1" t="s">
-        <v>161</v>
-      </c>
       <c r="G23" s="1" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="H23" s="1">
         <v>0</v>
@@ -2771,10 +2773,10 @@
         <v>52</v>
       </c>
       <c r="K23" s="1" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="L23" s="1" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="M23" s="1">
         <v>72</v>
@@ -2783,7 +2785,7 @@
         <v>0</v>
       </c>
       <c r="O23" s="1" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="P23" s="1">
         <v>1</v>
@@ -2815,25 +2817,25 @@
         <v>2025</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="D24" s="1">
         <v>27</v>
       </c>
       <c r="E24" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="G24" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="F24" s="1" t="s">
-        <v>165</v>
-      </c>
-      <c r="G24" s="1" t="s">
-        <v>166</v>
-      </c>
       <c r="H24" s="1" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="I24" s="1">
         <v>133</v>
@@ -2842,7 +2844,7 @@
         <v>66</v>
       </c>
       <c r="K24" s="1" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="L24" s="1">
         <v>3</v>
@@ -2854,7 +2856,7 @@
         <v>0</v>
       </c>
       <c r="O24" s="1" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="P24" s="1">
         <v>2</v>
@@ -2886,22 +2888,22 @@
         <v>2025</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="D25" s="4">
         <v>28</v>
       </c>
       <c r="E25" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="G25" s="4" t="s">
         <v>170</v>
-      </c>
-      <c r="F25" s="4" t="s">
-        <v>171</v>
-      </c>
-      <c r="G25" s="4" t="s">
-        <v>172</v>
       </c>
       <c r="H25" s="4">
         <v>0</v>
@@ -2913,10 +2915,10 @@
         <v>25</v>
       </c>
       <c r="K25" s="4" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="L25" s="4" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="M25" s="4">
         <v>39</v>
@@ -2925,7 +2927,7 @@
         <v>9</v>
       </c>
       <c r="O25" s="4" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="P25" s="4">
         <v>1</v>
@@ -2957,25 +2959,25 @@
         <v>2025</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="D26" s="4">
         <v>29</v>
       </c>
       <c r="E26" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="F26" s="4" t="s">
         <v>175</v>
       </c>
-      <c r="F26" s="4" t="s">
+      <c r="G26" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="H26" s="4" t="s">
         <v>177</v>
-      </c>
-      <c r="G26" s="4" t="s">
-        <v>178</v>
-      </c>
-      <c r="H26" s="4" t="s">
-        <v>179</v>
       </c>
       <c r="I26" s="4">
         <v>46</v>
@@ -2984,10 +2986,10 @@
         <v>23</v>
       </c>
       <c r="K26" s="4" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="L26" s="4" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="M26" s="4">
         <v>13</v>
@@ -2996,7 +2998,7 @@
         <v>0</v>
       </c>
       <c r="O26" s="4" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="P26" s="4">
         <v>5</v>
@@ -3028,25 +3030,25 @@
         <v>2025</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="D27" s="4">
         <v>30</v>
       </c>
       <c r="E27" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="F27" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="F27" s="4" t="s">
+      <c r="G27" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="H27" s="4" t="s">
         <v>183</v>
-      </c>
-      <c r="G27" s="4" t="s">
-        <v>184</v>
-      </c>
-      <c r="H27" s="4" t="s">
-        <v>185</v>
       </c>
       <c r="I27" s="4">
         <v>41</v>
@@ -3055,10 +3057,10 @@
         <v>20</v>
       </c>
       <c r="K27" s="4" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="L27" s="4" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="M27" s="4">
         <v>24</v>
@@ -3067,7 +3069,7 @@
         <v>1</v>
       </c>
       <c r="O27" s="4" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="P27" s="4">
         <v>28</v>
@@ -3099,25 +3101,25 @@
         <v>2025</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="D28" s="4">
         <v>31</v>
       </c>
       <c r="E28" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="F28" s="4" t="s">
         <v>188</v>
       </c>
-      <c r="F28" s="4" t="s">
+      <c r="G28" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="H28" s="4" t="s">
         <v>190</v>
-      </c>
-      <c r="G28" s="4" t="s">
-        <v>191</v>
-      </c>
-      <c r="H28" s="4" t="s">
-        <v>192</v>
       </c>
       <c r="I28" s="4">
         <v>34</v>
@@ -3126,10 +3128,10 @@
         <v>17</v>
       </c>
       <c r="K28" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="L28" s="4" t="s">
         <v>193</v>
-      </c>
-      <c r="L28" s="4" t="s">
-        <v>195</v>
       </c>
       <c r="M28" s="4">
         <v>12</v>
@@ -3138,7 +3140,7 @@
         <v>4</v>
       </c>
       <c r="O28" s="4" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="P28" s="4">
         <v>0</v>
@@ -3170,25 +3172,25 @@
         <v>2025</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="D29" s="4">
         <v>32</v>
       </c>
       <c r="E29" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F29" s="4" t="s">
         <v>196</v>
       </c>
-      <c r="F29" s="4" t="s">
+      <c r="G29" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="H29" s="4" t="s">
         <v>198</v>
-      </c>
-      <c r="G29" s="4" t="s">
-        <v>199</v>
-      </c>
-      <c r="H29" s="4" t="s">
-        <v>200</v>
       </c>
       <c r="I29" s="4">
         <v>37</v>
@@ -3197,10 +3199,10 @@
         <v>19</v>
       </c>
       <c r="K29" s="4" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="L29" s="4" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="M29" s="4">
         <v>20</v>
@@ -3209,7 +3211,7 @@
         <v>0</v>
       </c>
       <c r="O29" s="4" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="P29" s="4">
         <v>0</v>
@@ -3241,25 +3243,25 @@
         <v>2026</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="D30" s="4">
         <v>33</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="F30" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="G30" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="H30" s="4" t="s">
         <v>204</v>
-      </c>
-      <c r="G30" s="4" t="s">
-        <v>205</v>
-      </c>
-      <c r="H30" s="4" t="s">
-        <v>206</v>
       </c>
       <c r="I30" s="4">
         <v>91</v>
@@ -3268,10 +3270,10 @@
         <v>45</v>
       </c>
       <c r="K30" s="4" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="L30" s="4" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="M30" s="4">
         <v>10</v>
@@ -3280,7 +3282,7 @@
         <v>0</v>
       </c>
       <c r="O30" s="4" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="P30" s="4">
         <v>0</v>
@@ -3312,25 +3314,25 @@
         <v>2026</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="D31" s="4">
         <v>34</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="F31" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="G31" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="H31" s="4" t="s">
         <v>211</v>
-      </c>
-      <c r="G31" s="4" t="s">
-        <v>212</v>
-      </c>
-      <c r="H31" s="4" t="s">
-        <v>213</v>
       </c>
       <c r="I31" s="4">
         <v>79</v>
@@ -3339,10 +3341,10 @@
         <v>39</v>
       </c>
       <c r="K31" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="L31" s="4" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="M31" s="4">
         <v>15</v>
@@ -3351,7 +3353,7 @@
         <v>0</v>
       </c>
       <c r="O31" s="4" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="P31" s="4">
         <v>2</v>
@@ -3383,25 +3385,25 @@
         <v>2026</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="D32" s="4">
         <v>35</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="H32" s="4" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="I32" s="4">
         <v>128</v>
@@ -3410,10 +3412,10 @@
         <v>64</v>
       </c>
       <c r="K32" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="L32" s="4" t="s">
         <v>226</v>
-      </c>
-      <c r="L32" s="4" t="s">
-        <v>228</v>
       </c>
       <c r="M32" s="4">
         <v>41</v>
@@ -3422,7 +3424,7 @@
         <v>0</v>
       </c>
       <c r="O32" s="4" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="P32" s="4">
         <v>0</v>
@@ -3454,25 +3456,25 @@
         <v>2026</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="D33" s="4">
         <v>36</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="G33" s="4" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="H33" s="4" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="I33" s="4">
         <v>91</v>
@@ -3481,10 +3483,10 @@
         <v>45</v>
       </c>
       <c r="K33" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="L33" s="4" t="s">
         <v>227</v>
-      </c>
-      <c r="L33" s="4" t="s">
-        <v>229</v>
       </c>
       <c r="M33" s="4">
         <v>14</v>
@@ -3493,7 +3495,7 @@
         <v>0</v>
       </c>
       <c r="O33" s="4" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="P33" s="4">
         <v>5</v>
@@ -3525,25 +3527,25 @@
         <v>2026</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="D34" s="4">
         <v>37</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="G34" s="4" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="H34" s="4" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="I34" s="4">
         <v>53</v>
@@ -3555,7 +3557,7 @@
         <v>13</v>
       </c>
       <c r="L34" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="M34" s="4">
         <v>46</v>
@@ -3564,7 +3566,7 @@
         <v>2</v>
       </c>
       <c r="O34" s="4" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="P34" s="4">
         <v>1</v>
@@ -3596,22 +3598,22 @@
         <v>2026</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="D35" s="4">
         <v>38</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="G35" s="4" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="H35" s="4">
         <v>0</v>
@@ -3623,10 +3625,10 @@
         <v>51</v>
       </c>
       <c r="K35" s="4" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="L35" s="4" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="M35" s="4">
         <v>57</v>
@@ -3635,7 +3637,7 @@
         <v>0</v>
       </c>
       <c r="O35" s="4" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="P35" s="4">
         <v>0</v>

</xml_diff>